<commit_message>
Implement farmer CSV/XLSX bulk intake upload with row-level results
</commit_message>
<xml_diff>
--- a/docker/staff-ui/assets/farmer-import-template.xlsx
+++ b/docker/staff-ui/assets/farmer-import-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="BA2" t="inlineStr">
         <is>
-          <t>RAIN_FED</t>
+          <t>RAINFED</t>
         </is>
       </c>
       <c r="BB2" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="BU2" t="inlineStr">
         <is>
-          <t>MEHER</t>
+          <t>SUMMER</t>
         </is>
       </c>
       <c r="BV2" t="inlineStr">
@@ -2715,7 +2715,7 @@
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
-          <t>RAIN_FED</t>
+          <t>RAINFED</t>
         </is>
       </c>
     </row>
@@ -3181,13 +3181,13 @@
       <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Season</t>
+          <t>Season code from configured master data</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>MEHER</t>
+          <t>SUMMER</t>
         </is>
       </c>
     </row>
@@ -3273,7 +3273,7 @@
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Season</t>
+          <t>Season code from configured master data</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -3357,7 +3357,7 @@
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Season</t>
+          <t>Season code from configured master data</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>

</xml_diff>

<commit_message>
Fix bulk import menu and pinned platform compatibility; verify database flow
</commit_message>
<xml_diff>
--- a/docker/staff-ui/assets/farmer-import-template.xlsx
+++ b/docker/staff-ui/assets/farmer-import-template.xlsx
@@ -1276,7 +1276,7 @@
       </c>
       <c r="BU2" t="inlineStr">
         <is>
-          <t>SUMMER</t>
+          <t>MEHER</t>
         </is>
       </c>
       <c r="BV2" t="inlineStr">
@@ -3187,7 +3187,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>SUMMER</t>
+          <t>MEHER</t>
         </is>
       </c>
     </row>

</xml_diff>